<commit_message>
Update step logging format with bold step ID, data display, and location info
</commit_message>
<xml_diff>
--- a/Br.net login .xlsx
+++ b/Br.net login .xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\smart\OneDrive\Desktop\Chatgpt1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD24A4DE-CBD1-4339-A84A-06AD7F16D725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1D71283-0EA4-4301-9588-14AD1273AE74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{26A5588D-6DB4-4F1A-9805-B9C41FC223AD}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="73">
   <si>
     <t>TO BE EXECUTED</t>
   </si>
@@ -258,10 +258,13 @@
     <t>TS001TC001BR013</t>
   </si>
   <si>
-    <t>Enter User Name</t>
-  </si>
-  <si>
     <t>Start</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Enter User Name </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Enter Password </t>
   </si>
 </sst>
 </file>
@@ -830,7 +833,7 @@
         <v>25</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J3" s="4" t="s">
         <v>26</v>
@@ -853,7 +856,7 @@
         <v>25</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>29</v>
+        <v>72</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>30</v>
@@ -896,7 +899,7 @@
         <v>34</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>48</v>
@@ -979,7 +982,7 @@
         <v>34</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>48</v>

</xml_diff>